<commit_message>
itt and power test fix
</commit_message>
<xml_diff>
--- a/NonStopPower/NonStopPower.xlsx
+++ b/NonStopPower/NonStopPower.xlsx
@@ -9,6 +9,7 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overall" sheetId="1" state="visible" r:id="rId1"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Non-stop Power race 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Total Non-stop Power race 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -488,62 +489,66 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1455555</v>
+        <v>1522726</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Uli Diedrichsen</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr"/>
+          <t>Herbert Schwaninger Team DKS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>well:fair</t>
+        </is>
+      </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>40:28.282</t>
+          <t>40:31.371</t>
         </is>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
       <c r="I2" t="n">
-        <v>4.2</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>B</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>5707766</v>
+        <v>3022995</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Stefan Cornelius Bang</t>
+          <t>Jon Aramburu</t>
         </is>
       </c>
       <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr">
         <is>
-          <t>44:40.982</t>
+          <t>42:28.932</t>
         </is>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="I3" t="n">
-        <v>3.1</v>
+        <v>3.8</v>
       </c>
     </row>
     <row r="4">
@@ -554,35 +559,31 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>C</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>534616</v>
+        <v>4447312</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Steve Kenan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>GRIT</t>
-        </is>
-      </c>
+          <t>Ika Russ</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>46:23.384</t>
+          <t>43:52.315</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>102.402</v>
+        <v>0</v>
       </c>
       <c r="H4" t="n">
-        <v>225</v>
+        <v>289</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="5">
@@ -597,31 +598,245 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5609162</v>
+        <v>1969156</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Alan Robertson</t>
+          <t>David G&amp;oacute;mez</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Team Not Pogi</t>
+          <t>PETA-Z</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>43:25.746</t>
+          <t>45:09.561</t>
         </is>
       </c>
       <c r="G5" t="n">
         <v>0</v>
       </c>
       <c r="H5" t="n">
-        <v>233</v>
+        <v>213</v>
       </c>
       <c r="I5" t="n">
-        <v>3.3</v>
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>5473506</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Sebastian Peters</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>&amp;#129420; HCT &amp;#129420;</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>46:49.842</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>100.2809999999999</v>
+      </c>
+      <c r="H6" t="n">
+        <v>260</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>4426125</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>Pat McMahon - don't buy SRAM (CRAP)</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>48:11.214</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>181.6529999999998</v>
+      </c>
+      <c r="H7" t="n">
+        <v>187</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>369166</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Christopher Groening8750</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>49:23.537</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>253.9759999999997</v>
+      </c>
+      <c r="H8" t="n">
+        <v>227</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C9" t="n">
+        <v>4364981</v>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>eiichi &amp;#65339;ZEAL&amp;#65341;</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>49:24.267</t>
+        </is>
+      </c>
+      <c r="G9" t="n">
+        <v>254.7059999999997</v>
+      </c>
+      <c r="H9" t="n">
+        <v>205</v>
+      </c>
+      <c r="I9" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C10" t="n">
+        <v>1777812</v>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>HIDE K</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>50:39.373</t>
+        </is>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="n">
+        <v>166</v>
+      </c>
+      <c r="I10" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C11" t="n">
+        <v>3152611</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Pako Chaparro</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>53:58.692</t>
+        </is>
+      </c>
+      <c r="G11" t="n">
+        <v>199.319</v>
+      </c>
+      <c r="H11" t="n">
+        <v>163</v>
+      </c>
+      <c r="I11" t="n">
+        <v>2.1</v>
       </c>
     </row>
   </sheetData>
@@ -635,7 +850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -697,140 +912,415 @@
         </is>
       </c>
       <c r="C2" t="n">
-        <v>1455555</v>
+        <v>1522726</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Uli Diedrichsen</t>
+          <t>Herbert Schwaninger Team DKS</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>well:fair</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>40:31.371</t>
+        </is>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>261</v>
+      </c>
+      <c r="I2" t="n">
+        <v>4.1</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C3" t="n">
+        <v>3022995</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Jon Aramburu</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>42:28.932</t>
+        </is>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>263</v>
+      </c>
+      <c r="I3" t="n">
+        <v>3.8</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="C4" t="n">
+        <v>1969156</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>David G&amp;oacute;mez</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>PETA-Z</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>45:09.561</t>
+        </is>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="n">
+        <v>213</v>
+      </c>
+      <c r="I4" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C5" t="n">
+        <v>4426125</v>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Pat McMahon - don't buy SRAM (CRAP)</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>48:11.214</t>
+        </is>
+      </c>
+      <c r="G5" t="n">
+        <v>181.653</v>
+      </c>
+      <c r="H5" t="n">
+        <v>187</v>
+      </c>
+      <c r="I5" t="n">
+        <v>2.9</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C6" t="n">
+        <v>4364981</v>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>eiichi &amp;#65339;ZEAL&amp;#65341;</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>49:24.267</t>
+        </is>
+      </c>
+      <c r="G6" t="n">
+        <v>254.706</v>
+      </c>
+      <c r="H6" t="n">
+        <v>205</v>
+      </c>
+      <c r="I6" t="n">
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C7" t="n">
+        <v>1777812</v>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>HIDE K</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>50:39.373</t>
+        </is>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="n">
+        <v>166</v>
+      </c>
+      <c r="I7" t="n">
+        <v>2.6</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>E</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="C8" t="n">
+        <v>3152611</v>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>Pako Chaparro</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>53:58.692</t>
+        </is>
+      </c>
+      <c r="G8" t="n">
+        <v>199.319</v>
+      </c>
+      <c r="H8" t="n">
+        <v>163</v>
+      </c>
+      <c r="I8" t="n">
+        <v>2.1</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>pen</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>zwift_id</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>name</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>team_name</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>time</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>gap</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>avg_power</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>avg_wkg</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="C2" t="n">
+        <v>4447312</v>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Ika Russ</t>
         </is>
       </c>
       <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr">
         <is>
-          <t>40:28.282</t>
+          <t>43:52.315</t>
         </is>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>257</v>
+        <v>289</v>
       </c>
       <c r="I2" t="n">
-        <v>4.2</v>
+        <v>3.2</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>D</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>C</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>C</t>
-        </is>
-      </c>
       <c r="C3" t="n">
-        <v>5707766</v>
+        <v>5473506</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Stefan Cornelius Bang</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr"/>
+          <t>Sebastian Peters</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>&amp;#129420; HCT &amp;#129420;</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>44:40.982</t>
+          <t>46:49.842</t>
         </is>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>274</v>
+        <v>260</v>
       </c>
       <c r="I3" t="n">
-        <v>3.1</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>D</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>D</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>534616</v>
+        <v>369166</v>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Steve Kenan</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>GRIT</t>
-        </is>
-      </c>
+          <t>Christopher Groening8750</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr">
         <is>
-          <t>46:23.384</t>
+          <t>49:23.537</t>
         </is>
       </c>
       <c r="G4" t="n">
-        <v>102.402</v>
+        <v>153.695</v>
       </c>
       <c r="H4" t="n">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="I4" t="n">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>D</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>B</t>
-        </is>
-      </c>
-      <c r="C5" t="n">
-        <v>5609162</v>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>Alan Robertson</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>Team Not Pogi</t>
-        </is>
-      </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>43:25.746</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H5" t="n">
-        <v>233</v>
-      </c>
-      <c r="I5" t="n">
-        <v>3.3</v>
+        <v>2.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>